<commit_message>
Update Product.xlsx and logo image
</commit_message>
<xml_diff>
--- a/Product.xlsx
+++ b/Product.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="135" windowWidth="24855" windowHeight="12030"/>
+    <workbookView xWindow="240" yWindow="135" windowWidth="24855" windowHeight="12030" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="234">
   <si>
     <t>Sr No</t>
   </si>
@@ -355,6 +355,369 @@
   </si>
   <si>
     <t>Category</t>
+  </si>
+  <si>
+    <t>Moong Dal – Yellow</t>
+  </si>
+  <si>
+    <t>Urad Dal – White</t>
+  </si>
+  <si>
+    <t>Urad Gota / Whole Urad</t>
+  </si>
+  <si>
+    <t>Kabuli Chana / Chickpeas</t>
+  </si>
+  <si>
+    <t>Desi Chana / Kala Chana</t>
+  </si>
+  <si>
+    <t>Masoor Dal – Red</t>
+  </si>
+  <si>
+    <t>Whole Masoor</t>
+  </si>
+  <si>
+    <t>Masoor Dal – Black/Brown</t>
+  </si>
+  <si>
+    <t>Matar Dal / Split Peas</t>
+  </si>
+  <si>
+    <t>Green Peas – Dried</t>
+  </si>
+  <si>
+    <t>Yellow Peas – Dried</t>
+  </si>
+  <si>
+    <t>White Peas – Dried</t>
+  </si>
+  <si>
+    <t>Black-Eyed Peas / Lobia</t>
+  </si>
+  <si>
+    <t>Cowpea / Chawli</t>
+  </si>
+  <si>
+    <t>Rajma – Red Kidney Beans</t>
+  </si>
+  <si>
+    <t>Chitra Rajma</t>
+  </si>
+  <si>
+    <t>Jammu Rajma</t>
+  </si>
+  <si>
+    <t>Black Rajma</t>
+  </si>
+  <si>
+    <t>Soybean</t>
+  </si>
+  <si>
+    <t>Horse Gram / Kulthi Dal</t>
+  </si>
+  <si>
+    <t>Moth Dal / Moth Beans</t>
+  </si>
+  <si>
+    <t>Field Beans / Val Dal</t>
+  </si>
+  <si>
+    <t>Hyacinth Beans</t>
+  </si>
+  <si>
+    <t>Kulith</t>
+  </si>
+  <si>
+    <t>Adzuki Beans</t>
+  </si>
+  <si>
+    <t>Lima Beans</t>
+  </si>
+  <si>
+    <t>Navy Beans</t>
+  </si>
+  <si>
+    <t>Great Northern Beans</t>
+  </si>
+  <si>
+    <t>Borlotti Beans</t>
+  </si>
+  <si>
+    <t>Fava Beans / Broad Beans</t>
+  </si>
+  <si>
+    <t>Black Beans</t>
+  </si>
+  <si>
+    <t>Green Gram Split</t>
+  </si>
+  <si>
+    <t>Green Gram Whole</t>
+  </si>
+  <si>
+    <t>Bengal Gram Whole</t>
+  </si>
+  <si>
+    <t>Split Bengal Gram</t>
+  </si>
+  <si>
+    <t>Split Pigeon Peas</t>
+  </si>
+  <si>
+    <t>Mixed Dal / Panchmel Dal</t>
+  </si>
+  <si>
+    <t>Foxtail Millet (Kangni)</t>
+  </si>
+  <si>
+    <t>Little Millet (Kutki)</t>
+  </si>
+  <si>
+    <t>Kodo Millet (Kodon)</t>
+  </si>
+  <si>
+    <t>Barnyard Millet (Sanwa / Sama)</t>
+  </si>
+  <si>
+    <t>Proso Millet (Barri / Chena)</t>
+  </si>
+  <si>
+    <t>Browntop Millet (Korle)</t>
+  </si>
+  <si>
+    <t>Amaranth / Rajgira</t>
+  </si>
+  <si>
+    <t>Buckwheat / Kuttu</t>
+  </si>
+  <si>
+    <t>Job's Tears / Coix</t>
+  </si>
+  <si>
+    <t>Japanese Millet</t>
+  </si>
+  <si>
+    <t>Guinea Millet</t>
+  </si>
+  <si>
+    <t>Fonio</t>
+  </si>
+  <si>
+    <t>Brown Rice</t>
+  </si>
+  <si>
+    <t>Black Rice</t>
+  </si>
+  <si>
+    <t>Red Rice</t>
+  </si>
+  <si>
+    <t>Wild Rice</t>
+  </si>
+  <si>
+    <t>Whole Oats</t>
+  </si>
+  <si>
+    <t>Whole Barley</t>
+  </si>
+  <si>
+    <t>Whole Rye</t>
+  </si>
+  <si>
+    <t>Whole Buckwheat</t>
+  </si>
+  <si>
+    <t>Whole Quinoa</t>
+  </si>
+  <si>
+    <t>Whole Amaranth</t>
+  </si>
+  <si>
+    <t>Whole Triticale</t>
+  </si>
+  <si>
+    <t>Whole Spelt</t>
+  </si>
+  <si>
+    <t>Whole Einkorn</t>
+  </si>
+  <si>
+    <t>Whole Emmer / Farro</t>
+  </si>
+  <si>
+    <t>Whole Freekeh</t>
+  </si>
+  <si>
+    <t>Whole Teff</t>
+  </si>
+  <si>
+    <t>Whole Fonio</t>
+  </si>
+  <si>
+    <t>Whole Kamut / Khorasan Wheat</t>
+  </si>
+  <si>
+    <t>Whole Cornmeal / Whole Corn</t>
+  </si>
+  <si>
+    <t>Whole Durum Wheat</t>
+  </si>
+  <si>
+    <t>Whole Semolina Wheat / Hard Wheat</t>
+  </si>
+  <si>
+    <t>Whole Oat Groats</t>
+  </si>
+  <si>
+    <t>Whole Rye Grain</t>
+  </si>
+  <si>
+    <t>Whole Wheat Berries</t>
+  </si>
+  <si>
+    <t>Black Cardamom</t>
+  </si>
+  <si>
+    <t>Cloves</t>
+  </si>
+  <si>
+    <t>Cassia</t>
+  </si>
+  <si>
+    <t>Bay Leaf</t>
+  </si>
+  <si>
+    <t>Fenugreek Seeds</t>
+  </si>
+  <si>
+    <t>Mustard Seeds</t>
+  </si>
+  <si>
+    <t>Nigella Seeds (Kalonji)</t>
+  </si>
+  <si>
+    <t>Carom Seeds (Ajwain)</t>
+  </si>
+  <si>
+    <t>Celery Seeds</t>
+  </si>
+  <si>
+    <t>Dill Seeds</t>
+  </si>
+  <si>
+    <t>Poppy Seeds</t>
+  </si>
+  <si>
+    <t>Sesame Seeds</t>
+  </si>
+  <si>
+    <t>Kokum</t>
+  </si>
+  <si>
+    <t>Turmeric Powder</t>
+  </si>
+  <si>
+    <t>Red Chilli Powder</t>
+  </si>
+  <si>
+    <t>Coriander Powder</t>
+  </si>
+  <si>
+    <t>Cumin Powder</t>
+  </si>
+  <si>
+    <t>Black Pepper Powder</t>
+  </si>
+  <si>
+    <t>Dry Ginger Powder</t>
+  </si>
+  <si>
+    <t>Garlic Powder</t>
+  </si>
+  <si>
+    <t>Onion Powder</t>
+  </si>
+  <si>
+    <t>Fenugreek Powder</t>
+  </si>
+  <si>
+    <t>Fennel Powder</t>
+  </si>
+  <si>
+    <t>Cardamom Powder</t>
+  </si>
+  <si>
+    <t>Cinnamon Powder</t>
+  </si>
+  <si>
+    <t>Clove Powder</t>
+  </si>
+  <si>
+    <t>Nutmeg Powder</t>
+  </si>
+  <si>
+    <t>Mace Powder</t>
+  </si>
+  <si>
+    <t>Amchur Powder</t>
+  </si>
+  <si>
+    <t>Curry Powder</t>
+  </si>
+  <si>
+    <t>Garam Masala</t>
+  </si>
+  <si>
+    <t>Chaat Masala</t>
+  </si>
+  <si>
+    <t>Kitchen King Masala</t>
+  </si>
+  <si>
+    <t>Kashmiri Red Chilli</t>
+  </si>
+  <si>
+    <t>Guntur Red Chilli</t>
+  </si>
+  <si>
+    <t>Byadgi Chilli</t>
+  </si>
+  <si>
+    <t>Teja Chilli</t>
+  </si>
+  <si>
+    <t>Salem Turmeric</t>
+  </si>
+  <si>
+    <t>Erode Turmeric</t>
+  </si>
+  <si>
+    <t>Nizamabad Turmeric</t>
+  </si>
+  <si>
+    <t>Alleppey Green Cardamom</t>
+  </si>
+  <si>
+    <t>Malabar Black Pepper</t>
+  </si>
+  <si>
+    <t>Coorg Cardamom</t>
+  </si>
+  <si>
+    <t>Malabar Tamarind</t>
+  </si>
+  <si>
+    <t>Moong Dal – Green</t>
+  </si>
+  <si>
+    <t>Chana Dal</t>
+  </si>
+  <si>
+    <t>Catetory</t>
+  </si>
+  <si>
+    <t>Dal</t>
   </si>
 </sst>
 </file>
@@ -1873,9 +2236,643 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B121"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="34.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="B1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>231</v>
+      </c>
+      <c r="B7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" t="s">
+        <v>229</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>